<commit_message>
fixed kaad.transpose and transp_grad, added transpose with permutation
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44900F49-5009-46DB-9617-019817382C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385C679B-B86C-4E75-B933-D7C55EC1B3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="405" yWindow="6270" windowWidth="43200" windowHeight="23445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="405" yWindow="6270" windowWidth="21330" windowHeight="23445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="34">
   <si>
     <t>add</t>
   </si>
@@ -131,7 +131,13 @@
     <t>transpose</t>
   </si>
   <si>
-    <t>add shape checking for one input functions</t>
+    <t>make kaad functions safe</t>
+  </si>
+  <si>
+    <t>potentially add references (A,B) in kaad</t>
+  </si>
+  <si>
+    <t>comment functions in kaad</t>
   </si>
 </sst>
 </file>
@@ -765,7 +771,7 @@
         <v>12</v>
       </c>
       <c r="P6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -800,7 +806,7 @@
         <v>12</v>
       </c>
       <c r="P7" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -816,6 +822,9 @@
       <c r="N8" t="s">
         <v>12</v>
       </c>
+      <c r="P8" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M9" s="1" t="s">
@@ -824,6 +833,9 @@
       <c r="N9" t="s">
         <v>12</v>
       </c>
+      <c r="P9" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
@@ -850,7 +862,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:F2 P1:T3 V1:XFD4 F3:F9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576">
+  <conditionalFormatting sqref="D1:F2 P1:T3 V1:XFD4 F3:F9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576 P5 P8:P9">
     <cfRule type="cellIs" dxfId="14" priority="28" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
@@ -861,7 +873,7 @@
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:N4 A3:B7 G3:H7 D3:E10 J5:L10 M5:N12 D11:L11">
+  <conditionalFormatting sqref="J1:N4 A3:B7 G3:H7 D3:E10 J5:L10 M5:N12 D11:L11 P6:P7">
     <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
@@ -872,7 +884,7 @@
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3 P5:P9 A12:J15">
+  <conditionalFormatting sqref="P3 A12:J15">
     <cfRule type="cellIs" dxfId="8" priority="22" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>

</xml_diff>

<commit_message>
added tile operatin, updated todo
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C30D479-0DDE-4C1D-84AA-485930EE3660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A5C6FD-E5CF-4359-8E85-17E8229CA39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="405" yWindow="6270" windowWidth="21330" windowHeight="23445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31995" yWindow="8235" windowWidth="21330" windowHeight="23445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="36">
   <si>
     <t>add</t>
   </si>
@@ -138,6 +138,12 @@
   </si>
   <si>
     <t>comment functions in kaad</t>
+  </si>
+  <si>
+    <t>make more inputs of gradient functions const</t>
+  </si>
+  <si>
+    <t xml:space="preserve">make sure Recorder can run more than once </t>
   </si>
 </sst>
 </file>
@@ -703,6 +709,9 @@
       <c r="N4" t="s">
         <v>12</v>
       </c>
+      <c r="P4" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -842,7 +851,10 @@
         <v>20</v>
       </c>
       <c r="N10" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="P10" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -862,36 +874,36 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A12:J15">
+    <cfRule type="cellIs" dxfId="14" priority="22" operator="equal">
+      <formula>"n.a."</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="23" operator="equal">
+      <formula>"todo"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="24" operator="equal">
+      <formula>"done"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D1:F2 P1:T3 V1:XFD4 F3:F9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576">
-    <cfRule type="cellIs" dxfId="14" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="28" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="29" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="30" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:N4 A3:B7 G3:H7 D3:E10 P5:P9 J5:L10 M5:N12 D11:L11">
-    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
+  <conditionalFormatting sqref="J1:N4 A3:B7 G3:H7 P3:P9 D3:E10 J5:L10 M5:N12 D11:L11">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
-      <formula>"done"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P3 A12:J15">
-    <cfRule type="cellIs" dxfId="8" priority="22" operator="equal">
-      <formula>"n.a."</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="23" operator="equal">
-      <formula>"todo"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
added outer and dot operators
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E8FBB3-0B8F-41BA-819B-5068DBFCBF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62F1DB1-4E9D-4AE8-8DCA-AA56C5B241B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="2730" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t>scalar</t>
   </si>
@@ -130,6 +130,12 @@
   </si>
   <si>
     <t>todo</t>
+  </si>
+  <si>
+    <t>outer</t>
+  </si>
+  <si>
+    <t>dot</t>
   </si>
 </sst>
 </file>
@@ -185,7 +191,34 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="15">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD0CECE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -692,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
@@ -753,7 +786,7 @@
         <v>7</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N3" t="s">
         <v>34</v>
@@ -788,10 +821,10 @@
         <v>7</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="N4" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="P4" t="s">
         <v>26</v>
@@ -823,10 +856,10 @@
         <v>7</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="N5" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="P5" t="s">
         <v>31</v>
@@ -858,7 +891,7 @@
         <v>7</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="N6" t="s">
         <v>7</v>
@@ -893,7 +926,7 @@
         <v>7</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N7" t="s">
         <v>7</v>
@@ -925,7 +958,7 @@
         <v>7</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="N8" t="s">
         <v>7</v>
@@ -951,7 +984,7 @@
         <v>7</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
@@ -959,7 +992,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -967,7 +1000,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -975,54 +1008,81 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N14" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:B9 D3:E10 D11:L11">
-    <cfRule type="cellIs" dxfId="11" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="15" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="16" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F2 P1:T3 V1:XFD4 F3:H9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576">
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="13" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:N2 P3:P5 Q3:Q6 J3:L10 M3:N12 Q8:Q10 R9:T11 A12:J15">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+  <conditionalFormatting sqref="J1:N2 P3:P5 Q3:Q6 J3:L10 Q8:Q10 R9:T11 A12:J15">
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
+      <formula>"done"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:N14">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"n.a."</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"todo"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S8:T8">
-    <cfRule type="cellIs" dxfId="2" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="20" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="21" operator="equal">
       <formula>"todo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="22" operator="equal">
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update main.cpp and todo
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\kaad_cpp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62F1DB1-4E9D-4AE8-8DCA-AA56C5B241B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84F8ABC-1AF9-4150-9CBE-7C57278953D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="36">
   <si>
     <t>scalar</t>
   </si>
@@ -84,9 +84,6 @@
     <t>sum</t>
   </si>
   <si>
-    <t>make kaad functions safe</t>
-  </si>
-  <si>
     <t>power</t>
   </si>
   <si>
@@ -105,9 +102,6 @@
     <t>mean</t>
   </si>
   <si>
-    <t>comment functions in kaad</t>
-  </si>
-  <si>
     <t>max</t>
   </si>
   <si>
@@ -120,12 +114,6 @@
     <t>sub_matrix</t>
   </si>
   <si>
-    <t xml:space="preserve">make sure Recorder can run more than once </t>
-  </si>
-  <si>
-    <t>rework sum_acoss_dims_left with effstride</t>
-  </si>
-  <si>
     <t>tensordot</t>
   </si>
   <si>
@@ -136,6 +124,15 @@
   </si>
   <si>
     <t>dot</t>
+  </si>
+  <si>
+    <t>improve matmul cache locality</t>
+  </si>
+  <si>
+    <t>maybe reduce division in mean</t>
+  </si>
+  <si>
+    <t>declare args as restrict</t>
   </si>
 </sst>
 </file>
@@ -786,13 +783,13 @@
         <v>7</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N3" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="P3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -821,13 +818,13 @@
         <v>7</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P4" t="s">
         <v>34</v>
-      </c>
-      <c r="P4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -856,13 +853,13 @@
         <v>7</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="P5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -896,31 +893,28 @@
       <c r="N6" t="s">
         <v>7</v>
       </c>
-      <c r="P6" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="K7" t="s">
         <v>7</v>
@@ -934,25 +928,25 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="K8" t="s">
         <v>7</v>
@@ -966,19 +960,19 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H9" t="s">
         <v>7</v>
@@ -992,7 +986,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -1000,7 +994,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -1008,7 +1002,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N12" t="s">
         <v>7</v>
@@ -1016,7 +1010,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N13" t="s">
         <v>7</v>
@@ -1024,7 +1018,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N14" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
reworked unaryOps with new Nodes up to mean
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84F8ABC-1AF9-4150-9CBE-7C57278953D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750F4200-CF04-4E0D-B23F-ECED42D748AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t>scalar</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>declare args as restrict</t>
+  </si>
+  <si>
+    <t>maybe remove gradients that are just wrappers</t>
   </si>
 </sst>
 </file>
@@ -789,7 +792,7 @@
         <v>7</v>
       </c>
       <c r="P3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -824,7 +827,7 @@
         <v>7</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -859,7 +862,7 @@
         <v>30</v>
       </c>
       <c r="P5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -893,6 +896,9 @@
       <c r="N6" t="s">
         <v>7</v>
       </c>
+      <c r="P6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -1025,7 +1031,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:B9 D3:E10 D11:L11">
+  <conditionalFormatting sqref="A3:B9 D3:E10 D11:L11 P1:T2 Q3:T3 P4">
     <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
@@ -1036,7 +1042,7 @@
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:F2 P1:T3 V1:XFD4 F3:H9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576">
+  <conditionalFormatting sqref="D1:F2 V1:XFD4 F3:H9 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A16:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>
@@ -1047,7 +1053,7 @@
       <formula>"done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:N2 P3:P5 Q3:Q6 J3:L10 Q8:Q10 R9:T11 A12:J15">
+  <conditionalFormatting sqref="J1:N2 P4:P6 Q3:Q6 J3:L10 Q8:Q10 R9:T11 A12:J15">
     <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
       <formula>"n.a."</formula>
     </cfRule>

</xml_diff>

<commit_message>
added unary_sclarRhs for sum operator
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t xml:space="preserve">scalar</t>
   </si>
@@ -76,6 +76,9 @@
     <t xml:space="preserve">matmul</t>
   </si>
   <si>
+    <t xml:space="preserve">make sure pointwise operations work on transposed tensors</t>
+  </si>
+  <si>
     <t xml:space="preserve">divide</t>
   </si>
   <si>
@@ -83,6 +86,9 @@
   </si>
   <si>
     <t xml:space="preserve">batch_matmul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fix sum and mean operator</t>
   </si>
   <si>
     <t xml:space="preserve">power</t>
@@ -585,70 +591,76 @@
       <c r="N5" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="P5" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="Q5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="P6" s="0" t="s">
+        <v>22</v>
       </c>
       <c r="Q6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>7</v>
@@ -656,32 +668,32 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>7</v>
@@ -690,19 +702,19 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>7</v>
@@ -711,7 +723,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>7</v>
@@ -730,7 +742,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>7</v>
@@ -753,7 +765,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>7</v>
@@ -775,10 +787,10 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="M12" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -794,10 +806,10 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="M13" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -813,10 +825,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="M14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N14" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
perf: added recursive flex algorightm for mean_dim
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C65425-A970-4CE9-B715-C463AE7ABD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8852CF-12E0-4EB6-BFC9-4EF91BAD70D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9600" yWindow="5910" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="39">
   <si>
     <t>scalar</t>
   </si>
@@ -136,6 +136,12 @@
   </si>
   <si>
     <t>tensordot</t>
+  </si>
+  <si>
+    <t>remove Kernels::NullOp</t>
+  </si>
+  <si>
+    <t>remove unnecessary args from operation and gradient function calls</t>
   </si>
 </sst>
 </file>
@@ -936,6 +942,9 @@
       <c r="N8" t="s">
         <v>7</v>
       </c>
+      <c r="P8" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -961,6 +970,9 @@
       </c>
       <c r="N9" t="s">
         <v>7</v>
+      </c>
+      <c r="P9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: corrected issue with shapechecking transposed tensors in binOperator and fixed shapechecking in dot Operator
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43AC73FA-2E68-4835-B26C-E119E1BC4E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC46D3E3-AACF-4581-8F53-84E58BB36709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9600" yWindow="5910" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="38">
   <si>
     <t>scalar</t>
   </si>
@@ -57,9 +57,6 @@
     <t>dot</t>
   </si>
   <si>
-    <t>make sure pointwise operations work on transposed tensors</t>
-  </si>
-  <si>
     <t>subtract</t>
   </si>
   <si>
@@ -103,9 +100,6 @@
   </si>
   <si>
     <t>transpose</t>
-  </si>
-  <si>
-    <t>remove mul from end pointer</t>
   </si>
   <si>
     <t>min</t>
@@ -774,216 +768,210 @@
         <v>7</v>
       </c>
       <c r="P3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K4" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="N4" t="s">
         <v>7</v>
       </c>
       <c r="P4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="N5" t="s">
         <v>7</v>
       </c>
       <c r="P5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="N6" t="s">
         <v>7</v>
       </c>
       <c r="P6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K7" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="N7" t="s">
         <v>7</v>
       </c>
       <c r="P7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K8" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="N8" t="s">
         <v>7</v>
-      </c>
-      <c r="P8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H9" t="s">
         <v>7</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
-      </c>
-      <c r="P9" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -991,7 +979,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -999,26 +987,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="N12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="N13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="N14" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: removed Kernels::NullOp and replaced with Kernels::Null
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC46D3E3-AACF-4581-8F53-84E58BB36709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08186139-3994-4FF5-B2D0-365A7032A14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9600" yWindow="5910" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9120" yWindow="6300" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t>scalar</t>
   </si>
@@ -76,9 +76,6 @@
   </si>
   <si>
     <t>matmul</t>
-  </si>
-  <si>
-    <t>remove Kernels::NullOp</t>
   </si>
   <si>
     <t>divide</t>
@@ -803,7 +800,7 @@
         <v>7</v>
       </c>
       <c r="P4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -838,106 +835,103 @@
         <v>7</v>
       </c>
       <c r="P5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="N6" t="s">
         <v>7</v>
       </c>
       <c r="P6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K7" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="N7" t="s">
         <v>7</v>
-      </c>
-      <c r="P7" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="K8" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="N8" t="s">
         <v>7</v>
@@ -945,25 +939,25 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
@@ -971,7 +965,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -979,7 +973,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -987,26 +981,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N12" t="s">
         <v>34</v>
-      </c>
-      <c r="N12" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: added default operation and gradient pointers for Nodes where applicable
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08186139-3994-4FF5-B2D0-365A7032A14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2CDC6FA-717B-4962-869F-4D67D84A9FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9120" yWindow="6300" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="36">
   <si>
     <t>scalar</t>
   </si>
@@ -115,9 +115,6 @@
   </si>
   <si>
     <t>sum_dim</t>
-  </si>
-  <si>
-    <t>add default ops for Nodes</t>
   </si>
   <si>
     <t>mean</t>
@@ -869,9 +866,6 @@
       <c r="N6" t="s">
         <v>7</v>
       </c>
-      <c r="P6" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -965,7 +959,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -973,7 +967,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -981,26 +975,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" t="s">
         <v>33</v>
-      </c>
-      <c r="N12" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf: improved shape checking in sum and mean operators
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2CDC6FA-717B-4962-869F-4D67D84A9FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B224B2D6-C1CD-42AD-B671-D45419E8A0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9120" yWindow="6300" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4770" yWindow="10605" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="35">
   <si>
     <t>scalar</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>sum</t>
-  </si>
-  <si>
-    <t>use sum instead of sum_mean when nDims = 1</t>
   </si>
   <si>
     <t>max</t>
@@ -831,9 +828,6 @@
       <c r="N5" t="s">
         <v>7</v>
       </c>
-      <c r="P5" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -933,25 +927,25 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
@@ -959,7 +953,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -967,7 +961,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -975,26 +969,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" t="s">
         <v>32</v>
-      </c>
-      <c r="N12" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf: removed unnecessary arguments from sum_dim and mean_dim
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B224B2D6-C1CD-42AD-B671-D45419E8A0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D844FCBF-03DB-4DDF-97EE-13F36832D286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4770" yWindow="10605" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4770" yWindow="8235" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="34">
   <si>
     <t>scalar</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>batch_matmul</t>
-  </si>
-  <si>
-    <t>remove unnecessary args from operation and gradient function calls</t>
   </si>
   <si>
     <t>power</t>
@@ -793,9 +790,6 @@
       <c r="N4" t="s">
         <v>7</v>
       </c>
-      <c r="P4" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -863,31 +857,31 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="K7" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="N7" t="s">
         <v>7</v>
@@ -895,31 +889,31 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="K8" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N8" t="s">
         <v>7</v>
@@ -927,25 +921,25 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
@@ -953,7 +947,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -961,7 +955,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -969,26 +963,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N12" t="s">
         <v>31</v>
-      </c>
-      <c r="N12" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: added keepNDims flag for sum and mean
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D844FCBF-03DB-4DDF-97EE-13F36832D286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FB4CA6-E72A-473B-818D-65B75668CB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4770" yWindow="8235" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="33">
   <si>
     <t>scalar</t>
   </si>
@@ -64,9 +64,6 @@
   </si>
   <si>
     <t>outer</t>
-  </si>
-  <si>
-    <t>add keepnDims for sum and mean</t>
   </si>
   <si>
     <t>multiply</t>
@@ -755,9 +752,6 @@
       <c r="N3" t="s">
         <v>7</v>
       </c>
-      <c r="P3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -793,31 +787,31 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="N5" t="s">
         <v>7</v>
@@ -825,31 +819,31 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="K6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="N6" t="s">
         <v>7</v>
@@ -857,31 +851,31 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="K7" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="N7" t="s">
         <v>7</v>
@@ -889,31 +883,31 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="K8" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="N8" t="s">
         <v>7</v>
@@ -921,25 +915,25 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
@@ -947,7 +941,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
@@ -955,7 +949,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
@@ -963,26 +957,26 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N12" t="s">
         <v>30</v>
-      </c>
-      <c r="N12" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
style: added doxygen-style comments to all header files
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kaad_cpp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050AD857-BEA7-4D13-92ED-958596D24345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E6E698-F5E5-45C9-A22F-B5ECF32FF20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9315" yWindow="6675" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18015" yWindow="4530" windowWidth="43200" windowHeight="23445" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="46">
   <si>
     <t>scalar</t>
   </si>
@@ -57,6 +57,9 @@
     <t>dot</t>
   </si>
   <si>
+    <t>fix transpose</t>
+  </si>
+  <si>
     <t>subtract</t>
   </si>
   <si>
@@ -66,6 +69,9 @@
     <t>outer</t>
   </si>
   <si>
+    <t>maybe rename Unary::scalarRhs</t>
+  </si>
+  <si>
     <t>multiply</t>
   </si>
   <si>
@@ -75,6 +81,9 @@
     <t>matmul</t>
   </si>
   <si>
+    <t>maybe use std::transform</t>
+  </si>
+  <si>
     <t>divide</t>
   </si>
   <si>
@@ -84,6 +93,9 @@
     <t>batch_matmul</t>
   </si>
   <si>
+    <t>add loop for tensor with same shape and different stride</t>
+  </si>
+  <si>
     <t>power</t>
   </si>
   <si>
@@ -93,6 +105,9 @@
     <t>transpose</t>
   </si>
   <si>
+    <t>improve args of mean</t>
+  </si>
+  <si>
     <t>min</t>
   </si>
   <si>
@@ -102,28 +117,52 @@
     <t>sum</t>
   </si>
   <si>
+    <t>write main comment for kaad.h</t>
+  </si>
+  <si>
     <t>max</t>
   </si>
   <si>
     <t>sum_dim</t>
   </si>
   <si>
+    <t>write main page for doxygen</t>
+  </si>
+  <si>
     <t>mean</t>
   </si>
   <si>
+    <t>clear up transp kernel</t>
+  </si>
+  <si>
     <t>mean_dim</t>
   </si>
   <si>
+    <t>rename node input pointers to A and B</t>
+  </si>
+  <si>
     <t>tile</t>
   </si>
   <si>
     <t>todo</t>
   </si>
   <si>
+    <t>change matmul stride back to int *[3]</t>
+  </si>
+  <si>
     <t>slice</t>
   </si>
   <si>
     <t>tensordot</t>
+  </si>
+  <si>
+    <t>renew comments for Kernels</t>
+  </si>
+  <si>
+    <t>####</t>
+  </si>
+  <si>
+    <t>maybe add binary unary namespace to kernels</t>
   </si>
 </sst>
 </file>
@@ -686,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
@@ -752,220 +791,250 @@
       <c r="N3" t="s">
         <v>7</v>
       </c>
+      <c r="P3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H4" t="s">
         <v>7</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K4" t="s">
         <v>7</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N4" t="s">
         <v>7</v>
+      </c>
+      <c r="P4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H5" t="s">
         <v>7</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K5" t="s">
         <v>7</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N5" t="s">
         <v>7</v>
+      </c>
+      <c r="P5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H6" t="s">
         <v>7</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K6" t="s">
         <v>7</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="N6" t="s">
         <v>7</v>
+      </c>
+      <c r="P6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
         <v>7</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H7" t="s">
         <v>7</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="K7" t="s">
         <v>7</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="N7" t="s">
         <v>7</v>
+      </c>
+      <c r="P7" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
         <v>7</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="K8" t="s">
         <v>7</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="N8" t="s">
         <v>7</v>
+      </c>
+      <c r="P8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H9" t="s">
         <v>7</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="N9" t="s">
         <v>7</v>
+      </c>
+      <c r="P9" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M10" s="1" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="N10" t="s">
         <v>7</v>
+      </c>
+      <c r="P10" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M11" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="N11" t="s">
         <v>7</v>
+      </c>
+      <c r="P11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M12" s="1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="N12" t="s">
-        <v>30</v>
+        <v>39</v>
+      </c>
+      <c r="P12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M13" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="N13" t="s">
         <v>7</v>
@@ -973,10 +1042,23 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="M14" s="1" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="N14" t="s">
-        <v>30</v>
+        <v>39</v>
+      </c>
+      <c r="P14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P16" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: renamed unary::scalarRhs to unary::scalarOut
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="42">
   <si>
     <t xml:space="preserve">scalar</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t xml:space="preserve">dot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">maybe rename Unary::scalarRhs</t>
   </si>
   <si>
     <t xml:space="preserve">subtract</t>
@@ -237,16 +234,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -437,433 +438,507 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="5.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="5.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="B1" s="2"/>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="H1" s="2"/>
+      <c r="J1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1" t="s">
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="1"/>
-      <c r="P1" s="1" t="s">
+      <c r="N1" s="2"/>
+      <c r="P1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="H3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1"/>
-      <c r="M3" s="2" t="s">
+      <c r="K3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P3" s="0" t="s">
+      <c r="N3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1"/>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N4" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P4" s="0" t="s">
+      <c r="Q4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="2" t="s">
+      <c r="N5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P5" s="0" t="s">
+      <c r="Q5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="Q5" s="1"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1"/>
-      <c r="M6" s="2" t="s">
+      <c r="N6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="N6" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P6" s="0" t="s">
+      <c r="Q6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="Q6" s="1"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7" s="1"/>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N7" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P7" s="0" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L8" s="1"/>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N8" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P8" s="0" t="s">
+      <c r="Q8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="1"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="2" t="s">
+      <c r="N9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N9" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P9" s="0" t="s">
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="1"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="2" t="s">
+      <c r="N10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="N10" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="1"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="2" t="s">
+      <c r="N11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="N11" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P11" s="0" t="s">
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="M12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="1"/>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="M12" s="2" t="s">
+      <c r="N12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="N12" s="0" t="s">
+      <c r="P12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="P12" s="0" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="M13" s="3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="M13" s="2" t="s">
+      <c r="N13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="N13" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="P13" s="0" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="M14" s="3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="M14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N14" s="0" t="s">
-        <v>38</v>
+      <c r="N14" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="D1:F2 V1:XFD4 F3:H9 M3:N14 Z5:XFD7 AB8:XFD19 F10:I10 S12:T15 Z12:AA15 A18:AA19 A20:XFD22 A23:I32 O23:XFD32 A33:XFD1048576 A16:O17 Q16:AA17 P12">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">

</xml_diff>

<commit_message>
refactor: renamed in1 and in2 to A and B in Nodes
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="38">
   <si>
     <t xml:space="preserve">scalar</t>
   </si>
@@ -61,9 +61,6 @@
     <t xml:space="preserve">outer</t>
   </si>
   <si>
-    <t xml:space="preserve">maybe use std::transform</t>
-  </si>
-  <si>
     <t xml:space="preserve">multiply</t>
   </si>
   <si>
@@ -73,9 +70,6 @@
     <t xml:space="preserve">matmul</t>
   </si>
   <si>
-    <t xml:space="preserve">add loop for tensor with same shape and different stride</t>
-  </si>
-  <si>
     <t xml:space="preserve">divide</t>
   </si>
   <si>
@@ -85,9 +79,6 @@
     <t xml:space="preserve">batch_matmul</t>
   </si>
   <si>
-    <t xml:space="preserve">improve args of mean</t>
-  </si>
-  <si>
     <t xml:space="preserve">power</t>
   </si>
   <si>
@@ -95,9 +86,6 @@
   </si>
   <si>
     <t xml:space="preserve">transpose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rename node input pointers to A and B</t>
   </si>
   <si>
     <t xml:space="preserve">min</t>
@@ -567,173 +555,165 @@
       <c r="N4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P4" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P5" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P6" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P7" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="P7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="Q8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>7</v>
@@ -742,13 +722,13 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
@@ -764,7 +744,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>7</v>
@@ -787,13 +767,13 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
@@ -812,13 +792,13 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="M12" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -834,13 +814,13 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="M13" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -856,10 +836,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="M14" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
style: made node_matmul stride comment more accurate
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t xml:space="preserve">scalar</t>
   </si>
@@ -95,9 +95,6 @@
   </si>
   <si>
     <t xml:space="preserve">sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">change matmul stride back to int *[3]</t>
   </si>
   <si>
     <t xml:space="preserve">max</t>
@@ -694,26 +691,24 @@
       <c r="N8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P8" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>7</v>
@@ -722,13 +717,13 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
@@ -744,7 +739,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>7</v>
@@ -767,13 +762,13 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P11" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P11" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
@@ -792,13 +787,13 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="M12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N12" s="1" t="s">
+      <c r="P12" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -814,13 +809,13 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="M13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P13" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -836,10 +831,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="M14" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
style: reworked comments for kernels
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="33">
   <si>
     <t xml:space="preserve">scalar</t>
   </si>
@@ -103,31 +103,19 @@
     <t xml:space="preserve">sum_dim</t>
   </si>
   <si>
-    <t xml:space="preserve">replace Kenrels::Nullop in ops files with nullop in nodes.h</t>
-  </si>
-  <si>
     <t xml:space="preserve">mean</t>
   </si>
   <si>
     <t xml:space="preserve">mean_dim</t>
   </si>
   <si>
-    <t xml:space="preserve">####</t>
-  </si>
-  <si>
     <t xml:space="preserve">tile</t>
   </si>
   <si>
     <t xml:space="preserve">todo</t>
   </si>
   <si>
-    <t xml:space="preserve">renew comments for Kernels</t>
-  </si>
-  <si>
     <t xml:space="preserve">slice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">maybe add binary unary namespace to kernels</t>
   </si>
   <si>
     <t xml:space="preserve">tensordot</t>
@@ -722,9 +710,7 @@
       <c r="N9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P9" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
@@ -739,7 +725,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>7</v>
@@ -762,14 +748,12 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P11" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="P11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
@@ -787,14 +771,12 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="M12" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="P12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
@@ -809,14 +791,12 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="M13" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="P13" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="P13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
@@ -831,10 +811,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="M14" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>